<commit_message>
working on the internation rates for the retail side
</commit_message>
<xml_diff>
--- a/public/file/International Standard Rates Upload Template.xlsx
+++ b/public/file/International Standard Rates Upload Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\sonic_3\public\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62DB5763-0289-4D8F-8E91-3D71D2B22BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A10B6E8B-9CF2-4D4E-9C39-376ECA6175DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,9 +60,6 @@
     <t>Range Up</t>
   </si>
   <si>
-    <t>Zone 8a</t>
-  </si>
-  <si>
     <t>Zone 1</t>
   </si>
   <si>
@@ -70,6 +67,9 @@
   </si>
   <si>
     <t>Zone 13</t>
+  </si>
+  <si>
+    <t>Zone 8</t>
   </si>
 </sst>
 </file>
@@ -508,7 +508,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
@@ -529,7 +529,7 @@
         <v>6</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>7</v>
@@ -541,10 +541,10 @@
         <v>9</v>
       </c>
       <c r="N1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">

</xml_diff>